<commit_message>
DER, script e Quiz atualizado
</commit_message>
<xml_diff>
--- a/TI/BackLog.xlsx
+++ b/TI/BackLog.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db15eb02ce3cbac9/Desktop/Projeto Pessoal/TI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{D8170727-FCFE-4E68-87F6-E1B0A1388886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8963E976-C2E2-40C3-9841-E47D204627FC}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{D8170727-FCFE-4E68-87F6-E1B0A1388886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69133C49-CD0B-4AF0-9EE6-B5596600C19C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B3905394-6DEC-4D7F-9FCA-95C3FCBD5513}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="1368" windowWidth="17280" windowHeight="8880" xr2:uid="{B3905394-6DEC-4D7F-9FCA-95C3FCBD5513}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="105">
   <si>
     <t>REQUISITO</t>
   </si>
@@ -350,6 +351,9 @@
   </si>
   <si>
     <t>Banco de dados dos usuarios</t>
+  </si>
+  <si>
+    <t>Entregue</t>
   </si>
 </sst>
 </file>
@@ -501,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -527,17 +531,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -751,6 +758,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1103,16 +1114,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -1406,8 +1417,8 @@
       <c r="G12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>85</v>
+      <c r="H12" s="13" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1465,26 +1476,26 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="11" t="s">
+      <c r="C15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="9">
         <v>2</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H15" s="5" t="s">
@@ -1492,26 +1503,26 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="11" t="s">
+      <c r="C16" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F16" s="11">
+      <c r="F16" s="9">
         <v>2</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H16" s="5" t="s">
@@ -1519,26 +1530,26 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="11" t="s">
+      <c r="C17" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="10">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="9">
         <v>1</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H17" s="5" t="s">
@@ -1546,26 +1557,26 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="11" t="s">
+      <c r="C18" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="9">
         <v>2</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H18" s="5" t="s">
@@ -1573,26 +1584,26 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="11" t="s">
+      <c r="C19" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="9">
         <v>1</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H19" s="5" t="s">
@@ -1600,26 +1611,26 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="10">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="9">
         <v>1</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H20" s="5" t="s">
@@ -1627,26 +1638,26 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="10">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="9">
         <v>1</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H21" s="5" t="s">
@@ -1654,26 +1665,26 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="9">
         <v>1</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H22" s="5" t="s">
@@ -1681,26 +1692,26 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" s="11" t="s">
+      <c r="C23" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="9">
         <v>2</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H23" s="5" t="s">
@@ -1708,26 +1719,26 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" s="11" t="s">
+      <c r="C24" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="9">
         <v>2</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H24" s="5" t="s">
@@ -1735,26 +1746,26 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="11" t="s">
+      <c r="C25" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="9">
         <v>1</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H25" s="5" t="s">
@@ -1762,26 +1773,26 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="12">
+      <c r="E26" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="9">
         <v>1</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H26" s="5" t="s">
@@ -1789,26 +1800,26 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="11" t="s">
+      <c r="C27" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="9">
         <v>1</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H27" s="5" t="s">
@@ -1816,26 +1827,26 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="11" t="s">
+      <c r="C28" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F28" s="11">
+      <c r="F28" s="9">
         <v>2</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H28" s="5" t="s">
@@ -1843,26 +1854,26 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="9">
         <v>2</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H29" s="5" t="s">
@@ -1870,26 +1881,26 @@
       </c>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="9">
         <v>3</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H30" s="5" t="s">
@@ -1897,26 +1908,26 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="11" t="s">
+      <c r="C31" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="10">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="9">
         <v>1</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H31" s="5" t="s">
@@ -1924,26 +1935,26 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="9">
         <v>3</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H32" s="5" t="s">
@@ -1951,26 +1962,26 @@
       </c>
     </row>
     <row r="33" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="9">
         <v>3</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H33" s="5" t="s">
@@ -1978,26 +1989,26 @@
       </c>
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D34" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F34" s="11">
+      <c r="F34" s="9">
         <v>2</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H34" s="5" t="s">
@@ -2005,26 +2016,26 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C35" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D35" s="11" t="s">
+      <c r="C35" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="12">
+      <c r="E35" s="10">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="9">
         <v>2</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="G35" s="9" t="s">
         <v>40</v>
       </c>
       <c r="H35" s="5" t="s">

</xml_diff>

<commit_message>
Codigos da API que estavam encaminhando para o diretorio original da API e não estavam commitando minhas mudanças
</commit_message>
<xml_diff>
--- a/TI/BackLog.xlsx
+++ b/TI/BackLog.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db15eb02ce3cbac9/Desktop/Projeto Pessoal/Projeto-Pessoal-1-semestre/TI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{D8170727-FCFE-4E68-87F6-E1B0A1388886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{298A0151-D7EF-4381-A243-A4C51745C57E}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{D8170727-FCFE-4E68-87F6-E1B0A1388886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9F31808-38D4-4DA4-9F72-A80FD07D0559}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="2388" windowHeight="564" xr2:uid="{B3905394-6DEC-4D7F-9FCA-95C3FCBD5513}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="ESTADO">Tabela1[]</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="102">
   <si>
     <t>REQUISITO</t>
   </si>
@@ -283,9 +286,6 @@
     <t>Melhorar e finalizar toda e qualquer pendencia relacionada a documentação</t>
   </si>
   <si>
-    <t>PENDENTE</t>
-  </si>
-  <si>
     <t>Prévia da solução+apresentação</t>
   </si>
   <si>
@@ -340,7 +340,13 @@
     <t>Banco de dados dos usuarios</t>
   </si>
   <si>
-    <t>Entregue</t>
+    <t>ENTREGUE</t>
+  </si>
+  <si>
+    <t>ENTRGUE</t>
+  </si>
+  <si>
+    <t>E TREGUE</t>
   </si>
 </sst>
 </file>
@@ -371,16 +377,16 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFF00"/>
+      <sz val="28"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="28"/>
-      <color theme="1"/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -395,13 +401,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -500,12 +506,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -518,19 +518,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1093,37 +1099,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="A1" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="13" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1147,8 +1153,8 @@
       <c r="F3" s="1">
         <v>3</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>81</v>
+      <c r="G3" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1171,8 +1177,8 @@
       <c r="F4" s="1">
         <v>3</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>81</v>
+      <c r="G4" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1195,8 +1201,8 @@
       <c r="F5" s="1">
         <v>2</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>81</v>
+      <c r="G5" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1219,8 +1225,8 @@
       <c r="F6" s="1">
         <v>2</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>81</v>
+      <c r="G6" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1243,8 +1249,8 @@
       <c r="F7" s="1">
         <v>2</v>
       </c>
-      <c r="G7" s="5" t="s">
-        <v>81</v>
+      <c r="G7" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1267,8 +1273,8 @@
       <c r="F8" s="1">
         <v>2</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>81</v>
+      <c r="G8" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1291,8 +1297,8 @@
       <c r="F9" s="1">
         <v>2</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>81</v>
+      <c r="G9" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1315,13 +1321,13 @@
       <c r="F10" s="1">
         <v>2</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>81</v>
+      <c r="G10" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>28</v>
@@ -1339,8 +1345,8 @@
       <c r="F11" s="1">
         <v>3</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>81</v>
+      <c r="G11" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1363,8 +1369,8 @@
       <c r="F12" s="1">
         <v>3</v>
       </c>
-      <c r="G12" s="11" t="s">
-        <v>100</v>
+      <c r="G12" s="9" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1387,8 +1393,8 @@
       <c r="F13" s="1">
         <v>3</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>81</v>
+      <c r="G13" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1411,512 +1417,512 @@
       <c r="F14" s="1">
         <v>2</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>81</v>
+      <c r="G14" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="C15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="8">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="7">
         <v>2</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>81</v>
+      <c r="G15" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="7">
         <v>2</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>81</v>
+      <c r="G16" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="C17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="10">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="F17" s="9">
+      <c r="E17" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F17" s="7">
         <v>1</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>81</v>
+      <c r="G17" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="C18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="8">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="7">
         <v>2</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>81</v>
+      <c r="G18" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="C19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="7">
         <v>1</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>81</v>
+      <c r="G19" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="10">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="F20" s="9">
+      <c r="E20" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F20" s="7">
         <v>1</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>81</v>
+      <c r="G20" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="10">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="F21" s="9">
+      <c r="E21" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F21" s="7">
         <v>1</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>81</v>
+      <c r="G21" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="7">
         <v>1</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>81</v>
+      <c r="G22" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="C23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="7">
         <v>2</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>81</v>
+      <c r="G23" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="C24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F24" s="9">
+      <c r="F24" s="7">
         <v>2</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>81</v>
+      <c r="G24" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="C25" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="7">
         <v>1</v>
       </c>
-      <c r="G25" s="5" t="s">
-        <v>81</v>
+      <c r="G25" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="7">
         <v>1</v>
       </c>
-      <c r="G26" s="5" t="s">
-        <v>81</v>
+      <c r="G26" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="C27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F27" s="7">
         <v>1</v>
       </c>
-      <c r="G27" s="5" t="s">
-        <v>81</v>
+      <c r="G27" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="C28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E28" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F28" s="7">
         <v>2</v>
       </c>
-      <c r="G28" s="5" t="s">
-        <v>81</v>
+      <c r="G28" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="10">
+      <c r="E29" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="7">
         <v>2</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>81</v>
+      <c r="G29" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E30" s="10">
+      <c r="E30" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F30" s="9">
+      <c r="F30" s="7">
         <v>3</v>
       </c>
-      <c r="G30" s="5" t="s">
-        <v>81</v>
+      <c r="G30" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C31" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="C31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E31" s="10">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="F31" s="9">
+      <c r="E31" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F31" s="7">
         <v>1</v>
       </c>
-      <c r="G31" s="5" t="s">
-        <v>81</v>
+      <c r="G31" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E32" s="10">
+      <c r="E32" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F32" s="9">
+      <c r="F32" s="7">
         <v>3</v>
       </c>
-      <c r="G32" s="5" t="s">
-        <v>81</v>
+      <c r="G32" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E33" s="10">
+      <c r="E33" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F33" s="9">
+      <c r="F33" s="7">
         <v>3</v>
       </c>
-      <c r="G33" s="5" t="s">
-        <v>81</v>
+      <c r="G33" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="10">
+      <c r="E34" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F34" s="9">
+      <c r="F34" s="7">
         <v>2</v>
       </c>
-      <c r="G34" s="5" t="s">
-        <v>81</v>
+      <c r="G34" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="9" t="s">
+      <c r="C35" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E35" s="10">
+      <c r="E35" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="7">
         <v>2</v>
       </c>
-      <c r="G35" s="5" t="s">
-        <v>81</v>
+      <c r="G35" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1939,16 +1945,16 @@
       <c r="F36" s="1">
         <v>1</v>
       </c>
-      <c r="G36" s="8" t="s">
-        <v>81</v>
+      <c r="G36" s="6" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>9</v>
@@ -1963,16 +1969,16 @@
       <c r="F37" s="1">
         <v>1</v>
       </c>
-      <c r="G37" s="5" t="s">
-        <v>81</v>
+      <c r="G37" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>9</v>
@@ -1987,16 +1993,16 @@
       <c r="F38" s="1">
         <v>1</v>
       </c>
-      <c r="G38" s="5" t="s">
-        <v>81</v>
+      <c r="G38" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>9</v>
@@ -2011,16 +2017,16 @@
       <c r="F39" s="1">
         <v>1</v>
       </c>
-      <c r="G39" s="5" t="s">
-        <v>81</v>
+      <c r="G39" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>9</v>
@@ -2035,16 +2041,16 @@
       <c r="F40" s="1">
         <v>1</v>
       </c>
-      <c r="G40" s="5" t="s">
-        <v>81</v>
+      <c r="G40" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>13</v>
@@ -2059,16 +2065,16 @@
       <c r="F41" s="1">
         <v>2</v>
       </c>
-      <c r="G41" s="5" t="s">
-        <v>81</v>
+      <c r="G41" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>13</v>
@@ -2083,16 +2089,16 @@
       <c r="F42" s="1">
         <v>2</v>
       </c>
-      <c r="G42" s="5" t="s">
-        <v>81</v>
+      <c r="G42" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>9</v>
@@ -2107,16 +2113,16 @@
       <c r="F43" s="1">
         <v>1</v>
       </c>
-      <c r="G43" s="5" t="s">
-        <v>81</v>
+      <c r="G43" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>9</v>
@@ -2131,8 +2137,8 @@
       <c r="F44" s="1">
         <v>1</v>
       </c>
-      <c r="G44" s="7" t="s">
-        <v>81</v>
+      <c r="G44" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2147,7 +2153,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G3:G44">
+  <conditionalFormatting sqref="G28:G44 G3:G26">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"FINALIZADO"</formula>
     </cfRule>

</xml_diff>